<commit_message>
modify the blank row fault
</commit_message>
<xml_diff>
--- a/TSA_template.xlsx
+++ b/TSA_template.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\100_ShenJinLiang\Medini_Project\TSA_AutoGeneration\TSA_AutoGeneration\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\100_ShenJinLiang\Medini_Project\TSA_Demo\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE02D9FA-A178-4AEA-BADD-1A3E92F30A20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B2FB8E-635D-4630-B12C-6F104F805B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -110,7 +110,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="88">
   <si>
     <t>ASIL</t>
   </si>
@@ -374,6 +374,10 @@
   </si>
   <si>
     <t>GMS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BMS_3</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -951,7 +955,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.33203125" customWidth="1"/>
@@ -1158,45 +1162,77 @@
       <c r="J6" t="s">
         <v>22</v>
       </c>
-      <c r="K6" t="str">
-        <v>None</v>
+      <c r="K6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
+        <v>87</v>
+      </c>
+      <c r="D8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" t="s">
+        <v>79</v>
+      </c>
+      <c r="I8" t="s">
+        <v>86</v>
+      </c>
+      <c r="J8" t="s">
+        <v>22</v>
+      </c>
+      <c r="K8" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K6" xr:uid="{44180E71-E723-4CFC-82BE-038C6950C0B1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K6 K8" xr:uid="{44180E71-E723-4CFC-82BE-038C6950C0B1}">
       <formula1>INDIRECT("Table6[Task]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Direction:" prompt="Select the direction for the Port, eg. IN/OUT/INOUT" sqref="D2:D6" xr:uid="{845C6273-24E0-4AD9-A35F-F1D491FCE6DC}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Direction:" prompt="Select the direction for the Port, eg. IN/OUT/INOUT" sqref="D2:D6 D8" xr:uid="{845C6273-24E0-4AD9-A35F-F1D491FCE6DC}">
       <formula1>INDIRECT("Table2[Direction]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="ASIL:" prompt="Select the ASIL for the Port" sqref="G2:G6" xr:uid="{44543D41-2C31-4DE3-B1ED-34EE5C8B81DE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="ASIL:" prompt="Select the ASIL for the Port" sqref="G2:G6 G8" xr:uid="{44543D41-2C31-4DE3-B1ED-34EE5C8B81DE}">
       <formula1>INDIRECT("Table3[ASIL]")</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
   <extLst>
-    <ext uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E9A14E57-8855-4231-85AC-6B9A6950F590}">
           <x14:formula1>
             <xm:f>Library!$F$2:$F$10</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F6</xm:sqref>
+          <xm:sqref>F2:F6 F8</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Direction:" prompt="Select the direction for the Port, eg. IN/OUT/INOUT" xr:uid="{4E11AFF1-A6A4-4E85-8BF6-8F3A6B4D0522}">
           <x14:formula1>
             <xm:f>Library!$B$2:$B$4</xm:f>
           </x14:formula1>
-          <xm:sqref>D7:D9979</xm:sqref>
+          <xm:sqref>D7 D9:D9979</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="ASIL:" prompt="Select the ASIL for the Port" xr:uid="{702D29CA-F792-4571-B6D6-79F2DB6CFDC2}">
           <x14:formula1>
             <xm:f>Library!$D$2:$D$20</xm:f>
           </x14:formula1>
-          <xm:sqref>G7:G9979</xm:sqref>
+          <xm:sqref>G7 G9:G9979</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9D748ED0-1C83-4BE1-945A-8509F2CAD3E7}">
           <x14:formula1>
@@ -1350,7 +1386,7 @@
       </c>
       <c r="R4" s="4"/>
     </row>
-    <row r="5" spans="4:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:18" x14ac:dyDescent="0.3">
       <c r="D5" t="s">
         <v>32</v>
       </c>
@@ -1373,7 +1409,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="6" spans="4:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:18" x14ac:dyDescent="0.3">
       <c r="D6" t="s">
         <v>33</v>
       </c>
@@ -1390,7 +1426,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="4:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:18" x14ac:dyDescent="0.3">
       <c r="D7" t="s">
         <v>26</v>
       </c>
@@ -1407,7 +1443,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="4:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:18" x14ac:dyDescent="0.3">
       <c r="D8" t="s">
         <v>34</v>
       </c>
@@ -1421,7 +1457,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="4:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:18" x14ac:dyDescent="0.3">
       <c r="D9" t="s">
         <v>35</v>
       </c>
@@ -1435,7 +1471,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="4:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:18" x14ac:dyDescent="0.3">
       <c r="D10" t="s">
         <v>36</v>
       </c>
@@ -1443,7 +1479,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="4:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:18" x14ac:dyDescent="0.3">
       <c r="D11" t="s">
         <v>37</v>
       </c>
@@ -1451,7 +1487,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="4:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:18" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
         <v>3</v>
       </c>
@@ -1459,7 +1495,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="4:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:18" x14ac:dyDescent="0.3">
       <c r="D13" t="s">
         <v>1</v>
       </c>
@@ -1467,7 +1503,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="4:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:18" x14ac:dyDescent="0.3">
       <c r="D14" t="s">
         <v>38</v>
       </c>
@@ -1475,7 +1511,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="4:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:18" x14ac:dyDescent="0.3">
       <c r="D15" t="s">
         <v>39</v>
       </c>
@@ -1483,7 +1519,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:18" x14ac:dyDescent="0.3">
       <c r="D16" t="s">
         <v>11</v>
       </c>

</xml_diff>